<commit_message>
Sudah disalin ke Canva
</commit_message>
<xml_diff>
--- a/syahadah.xlsx
+++ b/syahadah.xlsx
@@ -1012,6 +1012,9 @@
     <xf numFmtId="0" fontId="20" fillId="36" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="20" fillId="37" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1023,9 +1026,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="37" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="42">
@@ -1490,41 +1490,41 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A1" s="11" t="s">
+      <c r="A1" s="12" t="s">
         <v>6</v>
       </c>
-      <c r="B1" s="12" t="s">
+      <c r="B1" s="13" t="s">
         <v>22</v>
       </c>
-      <c r="C1" s="13"/>
-      <c r="D1" s="13"/>
-      <c r="E1" s="13"/>
-      <c r="F1" s="13"/>
-      <c r="G1" s="13"/>
-      <c r="H1" s="13"/>
-      <c r="I1" s="14"/>
+      <c r="C1" s="14"/>
+      <c r="D1" s="14"/>
+      <c r="E1" s="14"/>
+      <c r="F1" s="14"/>
+      <c r="G1" s="14"/>
+      <c r="H1" s="14"/>
+      <c r="I1" s="15"/>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A2" s="11"/>
-      <c r="B2" s="11">
+      <c r="A2" s="12"/>
+      <c r="B2" s="12">
         <v>1</v>
       </c>
-      <c r="C2" s="11"/>
-      <c r="D2" s="11">
+      <c r="C2" s="12"/>
+      <c r="D2" s="12">
         <v>2</v>
       </c>
-      <c r="E2" s="11"/>
-      <c r="F2" s="11">
+      <c r="E2" s="12"/>
+      <c r="F2" s="12">
         <v>3</v>
       </c>
-      <c r="G2" s="11"/>
-      <c r="H2" s="11">
+      <c r="G2" s="12"/>
+      <c r="H2" s="12">
         <v>4</v>
       </c>
-      <c r="I2" s="11"/>
+      <c r="I2" s="12"/>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A3" s="11"/>
+      <c r="A3" s="12"/>
       <c r="B3" s="2" t="s">
         <v>23</v>
       </c>
@@ -1991,7 +1991,7 @@
       <c r="J1" s="10" t="s">
         <v>32</v>
       </c>
-      <c r="K1" s="15" t="s">
+      <c r="K1" s="11" t="s">
         <v>112</v>
       </c>
     </row>

</xml_diff>